<commit_message>
Con Law Midterm Q&A tab: explain only the right answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Con_Law_Outline_Week_8_with_Midterm_QA.xlsx
+++ b/Con_Law_Outline_Week_8_with_Midterm_QA.xlsx
@@ -12210,7 +12210,7 @@
       </c>
       <c r="C2" s="95" t="inlineStr">
         <is>
-          <t>Iredell accepted judicial review, but only to enforce the written Constitution, and only in a clear and urgent case. He rejected voiding laws for violating 'natural justice,' because natural-justice principles have no fixed standard and reasonable people disagree about them. D describes Justice Chase, who would let courts void laws contrary to 'first principles of the social compact' even without a specific textual provision. A is wrong because Iredell accepted the power. B invents a Tenth Amendment limit that neither Justice adopted.</t>
+          <t>Iredell accepted judicial review, but tied it to the written Constitution. A court may declare a legislative act void only when it clearly violates a particular constitutional provision, and only in a clear and urgent case. He refused to rest invalidation on 'natural justice,' because those principles have no fixed standard and the ablest people disagree about them.</t>
         </is>
       </c>
     </row>
@@ -12227,7 +12227,7 @@
       </c>
       <c r="C3" s="95" t="inlineStr">
         <is>
-          <t>Thomas argued the majority's holding (no concrete injury, so no Article III standing for most class members) didn't erase the statutory rights Congress created under the FCRA. Article III limits only federal courts. State courts aren't bound by federal justiciability rules, so plaintiffs can bring the same FCRA claims there. By closing the federal forum, the Court may have sent these class actions to state courts as the only forum, which is possibly worse for TransUnion. That's the 'pyrrhic victory.' A, B and C misdescribe the holding: it was a standing ruling, not a political-question or appellate-jurisdiction ruling, and Thomas's point wasn't about congressional override.</t>
+          <t>Thomas argued the majority's holding (no concrete injury, so no Article III standing for most class members) didn't erase the statutory rights Congress created under the FCRA. Article III limits only federal courts, and state courts aren't bound by federal justiciability rules. By closing the federal forum, the Court may have left state courts as the only forum for these class actions, and possibly a less favorable one for TransUnion. That's the 'pyrrhic victory.'</t>
         </is>
       </c>
     </row>
@@ -12244,7 +12244,7 @@
       </c>
       <c r="C4" s="95" t="inlineStr">
         <is>
-          <t>Seminole Tribe holds that Congress can't use its Article I powers, including the Commerce Clause, to abrogate state sovereign immunity. Allen v. Cooper applied the same rule to the Intellectual Property Clause. The exceptions are §5 of the Fourteenth Amendment (valid, congruent and proportional legislation) and the Bankruptcy Clause, where Katz found the states consented 'in the plan of the Convention.' A commerce-based trademark statute fits neither. A gets the rule backwards. B misapplies the plan-of-the-Convention reasoning, which Katz tied to bankruptcy. D is too broad because §5 abrogation is allowed.</t>
+          <t>Seminole Tribe holds that Congress can't use its Article I powers, including the Commerce Clause, to abrogate state sovereign immunity. Allen v. Cooper applied the same rule to the Intellectual Property Clause. The recognized routes are §5 of the Fourteenth Amendment and the Bankruptcy Clause (Katz, 'plan of the Convention'). A commerce-based trademark statute uses neither, so the abrogation is unconstitutional.</t>
         </is>
       </c>
     </row>
@@ -12263,7 +12263,7 @@
       </c>
       <c r="C5" s="95" t="inlineStr">
         <is>
-          <t>Under the aggregation principle (Wickard, Perez, Raich), Congress may regulate a class of activities that, taken together, substantially affects interstate commerce. Each individual instance doesn't need an interstate effect. Residential rentals are economic activity, and the rental market as a whole affects interstate commerce. Because the FAA reaches as far as the commerce power, the clause is likely enforceable. A and B look only at this one local transaction. C overstates the commerce power, which Lopez confirmed has limits and doesn't cover all intrastate commerce.</t>
+          <t>Under the aggregation principle (Wickard, Perez, Raich), Congress may regulate a class of economic activities that, taken together, substantially affects interstate commerce, even when an individual instance is local. Residential rentals are economic activity, and the rental market as a whole affects interstate commerce. Because the FAA reaches as far as the commerce power, the arbitration clause is likely enforceable.</t>
         </is>
       </c>
     </row>
@@ -12280,7 +12280,7 @@
       </c>
       <c r="C6" s="95" t="inlineStr">
         <is>
-          <t>A federal district court is bound by its own circuit's court of appeals (the Seventh Circuit for the Northern District of Illinois) and by the U.S. Supreme Court. District court decisions aren't binding precedent, even in the same district. The Illinois Supreme Court doesn't bind a federal court on a question of federal constitutional law. So only the Seventh Circuit, among the choices, is binding.</t>
+          <t>A federal district court is bound by the decisions of the court of appeals for its own circuit and by the U.S. Supreme Court. The Northern District of Illinois sits in the Seventh Circuit, so Seventh Circuit decisions bind it.</t>
         </is>
       </c>
     </row>
@@ -12314,7 +12314,7 @@
       </c>
       <c r="C8" s="95" t="inlineStr">
         <is>
-          <t>In Federalist No. 78, Hamilton argues the Constitution is fundamental law expressing the will of the people, superior to statutes reflecting the will of their agents. Where there's an irreconcilable variance, judges must prefer the Constitution to the statute. That doesn't make the judiciary superior to the legislature; it makes the people's will superior to both. A states the opposite. B invents an Article-by-Article split. D misreads the Founders' relationship to British legal traditions.</t>
+          <t>In Federalist No. 78, Hamilton argues the Constitution is fundamental law expressing the will of the people, superior to statutes, which reflect the will of the people's agents. When the two irreconcilably conflict, judges must prefer the Constitution. That doesn't make the judiciary superior to the legislature; it makes the people's will superior to both.</t>
         </is>
       </c>
     </row>
@@ -12331,7 +12331,7 @@
       </c>
       <c r="C9" s="95" t="inlineStr">
         <is>
-          <t>President Clinton responded by proposing to amend the Gun-Free School Zones Act to add a jurisdictional element, requiring that the firearm have moved in or otherwise affected interstate commerce. Congress did so in 1996 (amended 18 U.S.C. §922(q)), and courts later upheld the amended statute (e.g., United States v. Dorsey, 9th Cir. 2005).</t>
+          <t>President Clinton responded by proposing to amend the Gun-Free School Zones Act to add a jurisdictional element, requiring that the firearm have moved in or otherwise affected interstate commerce. That would bring the law within Congress's Commerce Clause authority. Congress enacted the amendment in 1996 (amended 18 U.S.C. §922(q)), and courts later upheld it (e.g., United States v. Dorsey, 9th Cir. 2005).</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="C10" s="95" t="inlineStr">
         <is>
-          <t>On a federal question, a state court is bound only by the U.S. Supreme Court (and by its own state's higher courts, which aren't among the choices). Lower federal courts, including the Central District of California and the Ninth Circuit, aren't above state courts. Their decisions are only persuasive in the Los Angeles County Superior Court, despite the geographic overlap.</t>
+          <t>On a question of federal law such as the First Amendment, a state court is bound by the U.S. Supreme Court, the final authority on federal constitutional questions. So a Supreme Court decision binds the Los Angeles County Superior Court.</t>
         </is>
       </c>
     </row>
@@ -12365,7 +12365,7 @@
       </c>
       <c r="C11" s="95" t="inlineStr">
         <is>
-          <t>Under Hans v. Louisiana, state sovereign immunity bars private damages suits against a nonconsenting state in federal court, whether the plaintiff is a citizen of that state or another. A damages claim against the program director that would be paid from the state treasury is really against the state (Edelman), so immunity applies. Congress didn't abrogate, and the statute is silent; abrogation requires an unmistakably clear statement and a valid source of power. B, C and D all treat the plaintiff's citizenship or the federal nature of the claim as decisive, but neither defeats immunity.</t>
+          <t>Under Hans v. Louisiana, state sovereign immunity bars private suits for damages against a nonconsenting state in federal court, including suits by the state's own citizens. A damages claim against the program director that would be paid from the state treasury is really a claim against the state (Edelman). The statute doesn't abrogate immunity, which requires an unmistakably clear statement and a valid source of power. So Illinois can claim sovereign immunity.</t>
         </is>
       </c>
     </row>
@@ -12385,7 +12385,7 @@
       </c>
       <c r="C12" s="95" t="inlineStr">
         <is>
-          <t>Clapper v. Amnesty International: the plaintiffs' fear of surveillance rested on a 'highly attenuated chain of possibilities.' They couldn't show their communications were or would be intercepted, so the injury wasn't 'certainly impending.' Any interception also might occur under some other authority, so it wasn't fairly traceable to §1881a. They can't manufacture standing by spending money to avoid a speculative harm, which is why D fails. A goes to the merits, not standing. C invents an attorney exception.</t>
+          <t>Clapper v. Amnesty International: a threatened injury must be 'certainly impending.' The plaintiffs' fear of interception rested on a speculative chain of possibilities, so they couldn't show an injury in fact. Any interception also might occur under some other authority, so it wasn't fairly traceable to §1881a. Costs they chose to incur to avoid a speculative harm can't create standing.</t>
         </is>
       </c>
     </row>
@@ -12419,7 +12419,7 @@
       </c>
       <c r="C14" s="95" t="inlineStr">
         <is>
-          <t>Marshall read §13 as conferring original jurisdiction to issue mandamus, which created the conflict with Article III. But a plausible alternative reading (often noted by commentators) is that §13 simply authorized the Court to issue writs of mandamus, warranted by the principles and usages of law, in cases already properly before it. That's a remedial power, not a jurisdictional grant. On that reading, there would have been no constitutional conflict and no need for judicial review.</t>
+          <t>Section 13 can plausibly be read as simply authorizing the Supreme Court to issue writs of mandamus, warranted by the principles and usages of law, in cases already properly before it. That's a remedial power, not a jurisdictional grant. On that reading, §13 wouldn't add to the Court's original jurisdiction, and there would be no conflict with Article III.</t>
         </is>
       </c>
     </row>
@@ -12440,7 +12440,7 @@
       </c>
       <c r="C15" s="95" t="inlineStr">
         <is>
-          <t>A plaintiff need not expose himself to arrest or prosecution to challenge a law that deters constitutionally protected conduct. A credible threat of prosecution is enough (Steffel v. Thompson). Smith was twice warned, his companion was actually arrested and charged, and the parties stipulated he might be arrested. That's a concrete, particularized and sufficiently imminent injury. B demands certainty, which isn't required. C misapplies TransUnion's history test, since threatened prosecution is a traditionally recognized harm. D confuses widespread risk with a generalized grievance; Smith is personally threatened.</t>
+          <t>A plaintiff need not expose himself to arrest or prosecution to challenge a law that deters constitutionally protected conduct. A credible threat of prosecution is enough (Steffel v. Thompson). Smith was twice warned, his companion was actually arrested and charged, and the parties stipulated he might be arrested if he returned. That's a concrete, particularized and sufficiently imminent injury.</t>
         </is>
       </c>
     </row>
@@ -12457,7 +12457,7 @@
       </c>
       <c r="C16" s="95" t="inlineStr">
         <is>
-          <t>In 1793, the Washington Administration asked the Justices for legal advice on questions of treaty construction and international law. The Justices declined, citing separation of powers and the courts' role as a court of last resort deciding actual cases. This established the precedent against federal advisory opinions. B, C and D attach the episode to doctrines that developed separately.</t>
+          <t>In 1793, the Washington Administration asked the Justices for legal advice on questions of treaty construction and international law. The Justices declined, citing separation of powers and the courts' role in deciding actual cases. This established the precedent that federal courts don't issue advisory opinions.</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="C17" s="95" t="inlineStr">
         <is>
-          <t>Brutus, a leading Anti-Federalist, warned that the Constitution's general, indefinite language (for example, 'necessary and proper' and 'general welfare') would be construed by judges to expand federal power. He argued this would gradually swallow and effectively abolish the state governments. Because judges would be independent and their constitutional rulings final, the legislature couldn't correct or control them. All three criticisms appear in Brutus.</t>
+          <t>Brutus, a leading Anti-Federalist, made each of these criticisms. The Constitution's general, indefinite language would be construed by judges in favor of federal power. That expansion would gradually swallow and effectively abolish the state governments. And because judges would be independent and their constitutional rulings final, the legislature couldn't control or correct the Supreme Court.</t>
         </is>
       </c>
     </row>
@@ -12491,7 +12491,7 @@
       </c>
       <c r="C18" s="95" t="inlineStr">
         <is>
-          <t>After Lopez, the most reliable way to keep a federal criminal statute within the Commerce Clause is a jurisdictional element requiring a case-by-case link to interstate commerce, such as a firearm that moved in interstate commerce. That's what Congress did when it amended §922(q), and courts upheld it (Dorsey). Findings and hearings help (C and B) but aren't dispositive; Morrison struck down VAWA's civil remedy despite extensive findings. A two-thirds majority (A) has no constitutional significance for enumerated power.</t>
+          <t>After Lopez, the most reliable way to keep a federal criminal statute within the Commerce Clause is a jurisdictional element requiring a case-specific link to interstate commerce, such as a firearm that moved in interstate commerce. Congress did exactly this when it amended §922(q) after Lopez, and courts upheld the amended statute (Dorsey).</t>
         </is>
       </c>
     </row>
@@ -12508,7 +12508,7 @@
       </c>
       <c r="C19" s="95" t="inlineStr">
         <is>
-          <t>Lopez identified three categories Congress may regulate: (1) the channels of interstate commerce, (2) the instrumentalities of interstate commerce and persons or things in it, and (3) activities that substantially affect interstate commerce. The effect must be substantial. The Court said formal findings are not required, although they can help a court evaluate the effect, so A and B are wrong. D is wrong because the Court decided the question on the merits.</t>
+          <t>Lopez identified three categories Congress may regulate under the Commerce Clause: (1) the channels of interstate commerce, (2) the instrumentalities of interstate commerce and persons or things in it, and (3) activities that substantially affect interstate commerce. For the third category, the effect must be substantial.</t>
         </is>
       </c>
     </row>
@@ -12526,7 +12526,7 @@
       </c>
       <c r="C20" s="95" t="inlineStr">
         <is>
-          <t>Perez v. United States (1971) upheld the federal loan-sharking (extortionate credit) statute as applied to purely intrastate transactions. Congress could regulate the whole class of activity because extortionate credit, as a class, affects interstate commerce. Lopez discussed Perez approvingly and didn't question it. Loan sharking is economic activity, unlike gun possession in Lopez. A relies on the 'costs of crime and education' reasoning Lopez rejected. C misstates Lopez: findings aren't required. D misreads both the Tenth Amendment and the case law.</t>
+          <t>Perez v. United States (1971) upheld the federal loan-sharking (extortionate credit) statute as applied to purely intrastate transactions. Congress could regulate the whole class of activity because extortionate credit, as a class, affects interstate commerce. Lopez cited Perez with approval and didn't question it, and loan sharking is economic activity. So a federal ban on loan sharking in schools fits within Perez.</t>
         </is>
       </c>
     </row>
@@ -12543,7 +12543,7 @@
       </c>
       <c r="C21" s="95" t="inlineStr">
         <is>
-          <t>Lopez didn't overrule any prior Commerce Clause case. Chief Justice Rehnquist treated Wickard, Perez and the other New Deal-era cases as still good law, and distinguished them on the ground that they involved economic activity, while gun possession in a school zone isn't economic.</t>
+          <t>Lopez didn't overrule any prior Commerce Clause case. Chief Justice Rehnquist treated Wickard, Perez and the other post-1937 cases as good law, and distinguished them on the ground that they involved economic activity, while possessing a gun in a school zone isn't economic.</t>
         </is>
       </c>
     </row>
@@ -12562,7 +12562,7 @@
       </c>
       <c r="C22" s="95" t="inlineStr">
         <is>
-          <t>The Court adopted Hamilton's view of the spending power (United States v. Butler; Helvering v. Davis). The power to tax and spend for the general welfare is a separate power, not limited to carrying out the other enumerated powers. Congress gets broad deference on what serves the general welfare, so a national museum is plainly within the power. B is Madison's narrower view, which the Court rejected. A misstates the test: national benefit doesn't require equal benefit to every state. D invents a location limit.</t>
+          <t>The Court adopted Hamilton's view of the spending power (United States v. Butler; Helvering v. Davis). The power to tax and spend for the general welfare is a separate power, not limited to carrying out the other enumerated powers in Article I, §8. Courts defer broadly to Congress's judgment about what serves the general welfare, so appropriating money for a national museum is within the power.</t>
         </is>
       </c>
     </row>
@@ -12579,7 +12579,7 @@
       </c>
       <c r="C23" s="95" t="inlineStr">
         <is>
-          <t>Mootness is standing set in a time frame: a live controversy must exist throughout the litigation, not just at filing. After graduation, with no intent to re-enroll, the plaintiff no longer has a personal stake in injunctive relief against the university's athletics program, so the claim became moot. She sought no damages that could keep it alive. A confuses ripeness (too early) with mootness (too late). D ignores that standing at filing isn't enough. C has no basis.</t>
+          <t>Mootness requires a live controversy throughout the litigation, not just when the suit is filed. Once the plaintiff graduated with no intent to re-enroll, she no longer had a personal stake in an injunction governing the university's athletics program. She sought no damages that could keep the case alive, so the claim became moot.</t>
         </is>
       </c>
     </row>
@@ -12596,7 +12596,7 @@
       </c>
       <c r="C24" s="95" t="inlineStr">
         <is>
-          <t>In Chisholm v. Georgia (1793), the Court held that Article III allowed a South Carolina citizen to sue Georgia in federal court without its consent, so Georgia had no immunity. The backlash produced the Eleventh Amendment (1795), which overturned Chisholm. B, C and D get the holding or the sequence backwards: Chisholm came before the Eleventh Amendment and rejected immunity.</t>
+          <t>In Chisholm v. Georgia (1793), the Court held that Article III allowed a South Carolina citizen to sue Georgia in federal court without its consent, so Georgia had no sovereign immunity. The decision provoked a strong backlash and led to the Eleventh Amendment (ratified 1795), which overturned Chisholm.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Con Law outline: add Week 2 readings fact bank tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Con_Law_Outline_Week_8_with_Midterm_QA.xlsx
+++ b/Con_Law_Outline_Week_8_with_Midterm_QA.xlsx
@@ -23,10 +23,12 @@
     <sheet name="Week 7 Class Notes" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Week 8 Reading Notes" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Week 1 Fact Bank" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Midterm questions &amp; answers" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Week 2 Fact Bank" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Midterm questions &amp; answers" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Week 1 Fact Bank'!$A$1:$F$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Week 2 Fact Bank'!$A$1:$F$157</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -17140,6 +17142,4741 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F157"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="96" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="96" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="C1" s="96" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="D1" s="96" t="inlineStr">
+        <is>
+          <t>Question (cover this column)</t>
+        </is>
+      </c>
+      <c r="E1" s="96" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+      <c r="F1" s="96" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Letter from the Justices to Washington (Aug. 8, 1793)</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>The Justices' letter of August 8, 1793: to whom, and responding to what?</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>To President George Washington, answering the "previous Question" in the letter the Secretary of State wrote at his direction on the 18th of the prior month (July 18, 1793).</t>
+        </is>
+      </c>
+      <c r="F2" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Letter from the Justices to Washington (Aug. 8, 1793)</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Signers</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Who signed the Justices' August 8, 1793 letter?</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>John Jay, James Wilson, John Blair, James Iredell ("Ja. Iredell") and William Paterson ("Wm Paterson").</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Letter from the Justices to Washington (Aug. 8, 1793)</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Reasons</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>What three considerations did the Justices say argue against "extrajudicially deciding" the questions?</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>(1) The lines of separation the Constitution draws between the three departments; (2) the departments being in certain respects checks on each other; (3) the Justices being "Judges of a court in the last Resort."</t>
+        </is>
+      </c>
+      <c r="F4" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Letter from the Justices to Washington (Aug. 8, 1793)</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Reasons</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>What textual argument did the Justices draw from the President's power to call for opinions?</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>The President's power to call on the Heads of Departments for opinions "seems to have been purposely as well as expressly limited to executive Departments" (so it does not reach the judges).</t>
+        </is>
+      </c>
+      <c r="F5" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Letter from the Justices to Washington (Aug. 8, 1793)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>What is the significance of the 1793 exchange of letters (Jefferson's request and the Justices' reply)?</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>The Justices declined to give the executive advice on legal questions outside a case: the origin of the federal courts' refusal to issue advisory opinions, grounded in separation of powers.</t>
+        </is>
+      </c>
+      <c r="F6" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Letter from the Justices to Washington (Aug. 8, 1793)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Tone</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>How did the Justices close their letter to Washington?</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>They "exceedingly regret" any embarrassment to his administration but trust his "Judgment," "Prudence, Decision and Firmness" will surmount every obstacle.</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Moore's Federal Practice (treatise)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>What is the Moore's reading, and where can it be found?</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>15 Moore's Federal Practice - Civil (Matthew Bender, 3d ed., 2025), "a leading treatise," available in hardcopy in the library and electronically on LEXIS.</t>
+        </is>
+      </c>
+      <c r="F8" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Moore's Federal Practice (treatise)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Why does the professor assign the Moore's sections?</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>As an overview of standing and (possibly) an introduction to the usefulness of a treatise; students need to be familiar with treatises in general and how to find things in them.</t>
+        </is>
+      </c>
+      <c r="F9" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Moore's Federal Practice (treatise)</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Sections</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Which four Moore's sections are assigned, and their titles?</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>§ 101.20 Focus of Standing Inquiry Is Who May Bring Suit; § 101.22 Historically, Standing Doctrine Has Included Both Constitutional and Prudential Requirements; § 101.23 Only One Plaintiff Need Have Standing; § 101.40 Standing Requires Injury-in-Fact.</t>
+        </is>
+      </c>
+      <c r="F10" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Moore's Federal Practice (treatise)</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Sections</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Per the Moore's section title, how many plaintiffs in a suit need standing?</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Only one (§ 101.23 "Only One Plaintiff Need Have Standing").</t>
+        </is>
+      </c>
+      <c r="F11" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Moore's Federal Practice (treatise)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Sections</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Per the Moore's section titles, what is the focus of the standing inquiry?</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>WHO may bring suit (§ 101.20).</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Citation and author of Massachusetts v. Mellon / Frothingham v. Mellon?</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>262 U.S. 447 (1923). Justice Sutherland delivered the opinion of the Court; the two cases were argued and decided together.</t>
+        </is>
+      </c>
+      <c r="F13" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>How did Massachusetts v. Mellon reach the Supreme Court?</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>As an ORIGINAL suit in the Supreme Court, brought by Massachusetts for herself and as representative of her citizens.</t>
+        </is>
+      </c>
+      <c r="F14" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>How did Frothingham v. Mellon reach the Supreme Court?</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>By appeal from the Court of Appeals of the District of Columbia, which affirmed the Supreme Court of the District's dismissal of her bill.</t>
+        </is>
+      </c>
+      <c r="F15" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>What statute was challenged in the Mellon cases, and what did it do?</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>The Maternity Act (Act of Nov. 23, 1921, 42 Stat. 224): appropriations for five years, apportioned among States that accept it, to reduce maternal and infant mortality and protect the health of mothers and infants; a federal bureau could withhold payments for improper spending.</t>
+        </is>
+      </c>
+      <c r="F16" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Who were the defendants in the Mellon cases?</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>The Secretary of the Treasury, the Chief of the Children's Bureau (Dept. of Labor), the Surgeon General (Public Health Service) and the Commissioner of Education; the last three formed the Board of Maternity and Infant Hygiene.</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Claims</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>What did Massachusetts claim in Massachusetts v. Mellon?</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>The Act usurped local self-government reserved by the Tenth Amendment, burdened industrial States unequally, and imposed an unconstitutional option: yield reserved rights or lose its share of the money. Massachusetts had NOT accepted the Act.</t>
+        </is>
+      </c>
+      <c r="F18" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Claims</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>What did Mrs. Frothingham claim?</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>As a federal taxpayer, the appropriations would increase her future taxes and so take her property without due process of law.</t>
+        </is>
+      </c>
+      <c r="F19" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Disposition of both Mellon cases?</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Both disposed of for want of jurisdiction, without reaching the merits.</t>
+        </is>
+      </c>
+      <c r="F20" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Why were the State's powers not invaded in Massachusetts v. Mellon?</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>The statute imposed no obligation; it simply extended an option the State was free to accept or reject. Congress's purpose to tempt may be frustrated "by the simple expedient of not yielding."</t>
+        </is>
+      </c>
+      <c r="F21" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Why did Massachusetts's claim fall outside the judicial power?</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>A State party gives original jurisdiction only for proceedings "of judicial cognizance." The naked contention that Congress usurped reserved powers by mere enactment is "political and not judicial in character."</t>
+        </is>
+      </c>
+      <c r="F22" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: which earlier case, by Justice Gray, refused a State's suit to enforce its own penal judgment against a citizen of another State?</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Wisconsin v. Pelican Insurance Co., 127 U.S. 265: the courts of no country will execute the penal laws of another.</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: in which cases did the Court keep original jurisdiction over State suits, and on what bases?</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Texas v. White, Florida v. Anderson, Alabama v. Burr (proprietary rights); Georgia v. Tennessee Copper Co. (dominion over air and soil); Missouri v. Holland (quasi-sovereign right to regulate taking of wild game); boundary disputes.</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: which cases denied State-suit jurisdiction?</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Mandamus by one State against another's Governor to surrender a fugitive (moral, not legal, duty); New Hampshire v. Louisiana / New York v. Louisiana (enforcing another State's bonds for assignors); Georgia v. Stanton (political/governmental questions).</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: why may a MUNICIPAL taxpayer sue when a federal taxpayer may not?</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>A municipal taxpayer's interest is "direct and immediate," resembling a stockholder's relation to a private corporation. A federal taxpayer's interest is shared with millions, "comparatively minute and indeterminable," and the effect on future taxation "remote, fluctuating and uncertain."</t>
+        </is>
+      </c>
+      <c r="F26" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: what consequence would follow if one federal taxpayer could sue?</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Every other taxpayer could sue over every appropriation act and statute requiring the outlay of public money; "the bare suggestion" of such a result, "with its attendant inconveniences," supports denying the suit.</t>
+        </is>
+      </c>
+      <c r="F27" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: what must the party invoking judicial review show?</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Not only that the statute is invalid but that he "has sustained or is immediately in danger of sustaining some direct injury" from its enforcement, "and not merely that he suffers in some indefinite way in common with people generally."</t>
+        </is>
+      </c>
+      <c r="F28" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Mellon: how does Sutherland describe the judicial power over unconstitutional statutes?</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>"We have no power per se to review and annul acts of Congress." It amounts to "little more than the negative power to disregard an unconstitutional enactment." In preventive relief the court enjoins not the statute's execution but the official's acts.</t>
+        </is>
+      </c>
+      <c r="F29" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Massachusetts v. Mellon / Frothingham v. Mellon (1923)</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Mellon's closing line about what deciding the case would mean?</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>It "would be not to decide a judicial controversy, but to assume a position of authority over the governmental acts of another and co-equal department, an authority which plainly we do not possess."</t>
+        </is>
+      </c>
+      <c r="F30" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen: citation and author?</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>392 U.S. 83 (1968). Chief Justice Warren delivered the opinion of the Court.</t>
+        </is>
+      </c>
+      <c r="F31" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>In what court did Flast v. Cohen begin?</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>The U.S. District Court for the Southern District of New York (suit to enjoin federal expenditures). The judgment below was REVERSED.</t>
+        </is>
+      </c>
+      <c r="F32" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>What statute and spending did the Flast plaintiffs challenge?</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Titles I and II of the Elementary and Secondary Education Act of 1965: federal funds used to finance instruction (reading, arithmetic, etc.) in religious schools and to buy textbooks and materials for them.</t>
+        </is>
+      </c>
+      <c r="F33" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>How many appellants were in Flast, and on what status did they rest standing?</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Seven, resting solely on their status as federal taxpayers ("each pay[s] income taxes of the United States").</t>
+        </is>
+      </c>
+      <c r="F34" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>Flast footnote 1: what additional allegation did the District Court treat as irrelevant?</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>That one appellant had children attending New York public schools. Appellants made no effort to rely on it.</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Claims</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Which constitutional clauses did the Flast plaintiffs invoke?</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>The Establishment and Free Exercise Clauses of the First Amendment (compulsory taxation for religious purposes).</t>
+        </is>
+      </c>
+      <c r="F36" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>How did Flast characterize Frothingham's 45-year effect?</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>An "impenetrable barrier" to suits against Acts of Congress by individuals asserting only the interest of federal taxpayers.</t>
+        </is>
+      </c>
+      <c r="F37" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Flast: what were the competing readings of Frothingham?</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>The Government: a constitutional rule (Article III and separation of powers). Appellants: a mere policy of judicial self-restraint. The Court: the opinion "can be read to support either position." Commentators (n.6) prevailingly saw a nonconstitutional rule of self-restraint.</t>
+        </is>
+      </c>
+      <c r="F38" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Flast: what quip did the Court make about why Mrs. Frothingham lost?</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Its reasoning suggests she "was denied standing not because she was a taxpayer but because her tax bill was not large enough."</t>
+        </is>
+      </c>
+      <c r="F39" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>Flast: what modern developments undercut Frothingham's policy concerns?</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>Corporate taxpayers with federal tax liabilities of hundreds of millions of dollars; and class actions and joinder under the Federal Rules of Civil Procedure, adopted after Frothingham.</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>Flast: what "quality" did the Court ascribe to the words "cases" and "controversies"?</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>An "iceberg quality": surface simplicity concealing "submerged complexities which go to the very heart of our constitutional form of government."</t>
+        </is>
+      </c>
+      <c r="F41" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Justiciability</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>Flast: the two limitations embodied in "cases" and "controversies"?</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>(1) Questions presented in an adversary context and in a form historically viewed as capable of judicial resolution; (2) the judiciary's role in a tripartite allocation of power, so courts do not intrude on the other branches. "Justiciability" is the term for this dual limitation.</t>
+        </is>
+      </c>
+      <c r="F42" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>Flast: why look to the substantive issues when deciding standing?</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>To decide whether there is a "logical nexus between the status asserted and the claim sought to be adjudicated" (e.g., standing differs for Establishment and Free Exercise claims).</t>
+        </is>
+      </c>
+      <c r="F43" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>Flast two-part nexus test: first nexus?</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>A logical link between taxpayer status and the type of enactment attacked: only exercises of congressional power under the taxing and spending clause of Art. I, § 8. Not an incidental expenditure in administering an essentially regulatory statute.</t>
+        </is>
+      </c>
+      <c r="F44" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>Flast two-part nexus test: second nexus?</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>A nexus between taxpayer status and the precise nature of the infringement: the enactment exceeds SPECIFIC constitutional limitations on the taxing and spending power, not merely that it is generally beyond Art. I, § 8 powers.</t>
+        </is>
+      </c>
+      <c r="F45" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>Flast: which clause is identified as a specific limit on the taxing and spending power?</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>The Establishment Clause. Whether other specific limitations exist "can be determined only in the context of future cases."</t>
+        </is>
+      </c>
+      <c r="F46" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>How did Flast reconcile its result with Frothingham?</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Frothingham met the first nexus (spending program) but not the second: she alleged Congress exceeded its general Art. I, § 8 powers and invaded State prerogatives (Tenth Amendment), and the Fifth Amendment Due Process Clause does not protect against tax increases.</t>
+        </is>
+      </c>
+      <c r="F47" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>Flast holding?</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>A taxpayer has Article III standing when he alleges congressional action under the taxing and spending clause violates constitutional provisions that restrict that power; the Flast appellants satisfied both nexuses. No view on the merits.</t>
+        </is>
+      </c>
+      <c r="F48" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>Flast: what does a taxpayer who fails the test seek to do?</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>"employ a federal court as a forum in which to air his generalized grievances about the conduct of government or the allocation of power in the Federal System."</t>
+        </is>
+      </c>
+      <c r="F49" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Concurrence</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>Justice Douglas's concurrence in Flast?</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>He joined, but thought the test not "durable" (for reasons stated by Harlan); it would erode and lead to Frothingham's demise, so it would be wise "to be rid of Frothingham here and now."</t>
+        </is>
+      </c>
+      <c r="F50" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Flast v. Cohen (1968)</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>Justice Harlan's dissent in Flast?</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>The end result of Frothingham was correct even though he does not accept all its reasoning; he cannot accept the substituted standing doctrine, which "rests on premises that do not withstand analysis."</t>
+        </is>
+      </c>
+      <c r="F51" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton: citation, author and lineup?</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>405 U.S. 727 (1972). Justice Stewart for the Court, joined by Burger, White and Marshall. Dissents: Douglas, Brennan, Blackmun. Powell and Rehnquist took no part.</t>
+        </is>
+      </c>
+      <c r="F52" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>Where is Mineral King, and what is its status?</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>A valley in the Sierra Nevada, Tulare County, California, adjacent to Sequoia National Park; part of Sequoia National Forest since 1926 and a national game refuge by special Act of Congress.</t>
+        </is>
+      </c>
+      <c r="F53" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: who won the Forest Service bidding, and what did it get?</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>Walt Disney Enterprises, Inc., chosen from six bidders after a 1965 prospectus; it got a three-year permit to conduct surveys and explorations for a master plan.</t>
+        </is>
+      </c>
+      <c r="F54" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: the final Disney plan's numbers?</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>Approved January 1969: a $35 million complex for 14,000 visitors daily, on 80 acres of valley floor under a 30-year use permit; ski lifts etc. under a revocable special-use permit.</t>
+        </is>
+      </c>
+      <c r="F55" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: what access and utility facilities would cross Sequoia National Park?</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>A 20-mile highway to be built by the State of California, and a high-voltage power line (66,000 volts, per Blackmun). Both needed Interior Department approval.</t>
+        </is>
+      </c>
+      <c r="F56" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: when and where was suit filed, and under what statute?</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>June 1969, U.S. District Court for the Northern District of California; § 10 of the Administrative Procedure Act (5 U.S.C. § 702).</t>
+        </is>
+      </c>
+      <c r="F57" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: what did the District Court and Ninth Circuit do?</t>
+        </is>
+      </c>
+      <c r="E58" s="14" t="inlineStr">
+        <is>
+          <t>After two days of hearings the District Court granted a preliminary injunction and upheld standing. The Ninth Circuit reversed, finding no allegation members were affected other than displeasure. The Supreme Court affirmed.</t>
+        </is>
+      </c>
+      <c r="F58" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>How did the Sierra Club describe itself in paragraph 3 of its complaint?</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>A California nonprofit based in San Francisco since 1892; about 78,000 members nationally, about 27,000 in the Bay Area, with "a special interest in the conservation and the sound maintenance" of parks, refuges and forests.</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>APA § 10 (5 U.S.C. § 702) text?</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>"A person suffering legal wrong because of agency action, or adversely affected or aggrieved by agency action within the meaning of a relevant statute, is entitled to judicial review thereof."</t>
+        </is>
+      </c>
+      <c r="F60" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>What test did Data Processing Service v. Camp and Barlow v. Collins set for APA standing?</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>"Injury in fact" plus an interest "arguably within the zone of interests to be protected or regulated" by the statute. Data Processing: competitors hurt by a Comptroller ruling letting banks do data processing. Barlow: tenant farmers vs. Agriculture regulations.</t>
+        </is>
+      </c>
+      <c r="F61" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club footnote 3: three things Congress cannot authorize Article III courts to do?</t>
+        </is>
+      </c>
+      <c r="E62" s="14" t="inlineStr">
+        <is>
+          <t>Render advisory opinions (Muskrat v. United States), entertain "friendly" suits (United States v. Johnson), or resolve "political questions" (Luther v. Borden).</t>
+        </is>
+      </c>
+      <c r="F62" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: is aesthetic or environmental harm an injury in fact?</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>Yes, it may be; interests shared by the many are no less deserving. "But the 'injury in fact' test requires more than an injury to a cognizable interest. It requires that the party seeking review be himself among the injured."</t>
+        </is>
+      </c>
+      <c r="F63" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: why did the Club lack standing?</t>
+        </is>
+      </c>
+      <c r="E64" s="14" t="inlineStr">
+        <is>
+          <t>It failed to allege that it or its members used Mineral King for any purpose, or would be affected in their activities or pastimes by the development. A mere "interest in a problem" is not enough.</t>
+        </is>
+      </c>
+      <c r="F64" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club footnote 8: what did the Wilderness Society amici assert, and why didn't it matter?</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>That the Club ran camping trips to Mineral King and members used it. These allegations weren't in the pleadings or raised below, and the Club declined to rely on individualized interest. It could still seek to amend under Rule 15.</t>
+        </is>
+      </c>
+      <c r="F65" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club: what would be undermined by allowing suits by those who "seek to do no more than vindicate their own value preferences"?</t>
+        </is>
+      </c>
+      <c r="E66" s="14" t="inlineStr">
+        <is>
+          <t>The goal of putting the decision to seek review "in the hands of those who have a direct stake in the outcome."</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>Justice Douglas's dissent in Sierra Club?</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>Standing should be conferred on environmental objects (inanimate objects about to be despoiled) to sue in their own name for their own preservation.</t>
+        </is>
+      </c>
+      <c r="F67" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>Justice Blackmun's dissent in Sierra Club: his opening question?</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>"Must our law be so rigid and our procedural concepts so inflexible that we render ourselves helpless when the existing methods and the traditional concepts do not quite fit...?"</t>
+        </is>
+      </c>
+      <c r="F68" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun in Sierra Club: what does he predict, and how big was the project?</t>
+        </is>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>The 35.3-million-dollar complex, "over 10 times greater than the Forest Service's suggested minimum," will proceed, opposition will recede, and Mineral King will be defaced.</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun's two alternatives in Sierra Club?</t>
+        </is>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>(1) Reverse and approve the District Court's standing and relief on condition the Club promptly amend its complaint; or (2) an "imaginative expansion" of standing to let bona fide environmental organizations like the Club litigate.</t>
+        </is>
+      </c>
+      <c r="F70" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>Sierra Club v. Morton (1972)</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun in Sierra Club: the "dual permit" issue?</t>
+        </is>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
+          <t>Whether the "dual permit" device avoided the 80-acre "recreation and resort" limit of 16 U.S.C. § 497 (expanded in 1956 from an old five-acre limit), an issue apparently never litigated.</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson: citation, author and lineup?</t>
+        </is>
+      </c>
+      <c r="E72" s="14" t="inlineStr">
+        <is>
+          <t>418 U.S. 166 (1974). Chief Justice Burger for the Court, joined by White, Blackmun, Powell and Rehnquist. Powell concurred. Dissents: Douglas; Brennan; Stewart joined by Marshall.</t>
+        </is>
+      </c>
+      <c r="F72" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
+        <is>
+          <t>What statute and clause were at issue in Richardson?</t>
+        </is>
+      </c>
+      <c r="E73" s="14" t="inlineStr">
+        <is>
+          <t>The Central Intelligence Agency Act of 1949 (secret CIA expenditures) challenged under Art. I, § 9, cl. 7: "a regular Statement and Account of the Receipts and Expenditures of all public Money shall be published from time to time" (Statement and Account / Accounts Clause).</t>
+        </is>
+      </c>
+      <c r="F73" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>In what capacities did Richardson claim standing?</t>
+        </is>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
+        <is>
+          <t>As a federal taxpayer (the question on certiorari); his complaint also called him "a member of the electorate, and a loyal citizen."</t>
+        </is>
+      </c>
+      <c r="F74" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>Richardson holding?</t>
+        </is>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>No standing; reversed. His claim fails the Flast taxpayer test and is a "generalized grievance": the impact on him is "plainly undifferentiated and 'common to all members of the public.'" (quoting Ex parte Levitt).</t>
+        </is>
+      </c>
+      <c r="F75" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
+        <is>
+          <t>What injury did Richardson assert?</t>
+        </is>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>Without detailed CIA expenditure information he could not intelligently follow Congress and the Executive or properly fulfill his obligations as a voter.</t>
+        </is>
+      </c>
+      <c r="F76" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>Richardson: what would allowing such suits imply the Founders intended?</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>"something in the nature of an Athenian democracy or a New England town meeting to oversee the conduct of the National Government by means of lawsuits in federal courts."</t>
+        </is>
+      </c>
+      <c r="F77" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D78" s="14" t="inlineStr">
+        <is>
+          <t>Richardson: if no one can sue, where does the issue go?</t>
+        </is>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>To the surveillance of Congress and ultimately the political process: representatives answerable at stated periods of two, four and six years. "Lack of standing" does not impair his right to assert his views "in the political forum or at the polls."</t>
+        </is>
+      </c>
+      <c r="F78" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>Concurrence</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>Justice Powell's concurrence in Richardson?</t>
+        </is>
+      </c>
+      <c r="E79" s="14" t="inlineStr">
+        <is>
+          <t>He would go further and abandon the Flast two-part "nexus" test (not a reliable indicator), but would not overrule Flast on its facts, since taxpayer standing in Establishment Clause cases is settled.</t>
+        </is>
+      </c>
+      <c r="F79" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>Justice Douglas's dissent in Richardson: key line?</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
+        <is>
+          <t>"The sovereign in this Nation is the people, not the bureaucracy." Without the statement of accounts, sovereignty becomes "an empty symbol and a secret bureaucracy is allowed to run our affairs." He would affirm the Court of Appeals.</t>
+        </is>
+      </c>
+      <c r="F80" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>Justice Stewart's dissent in Richardson (joined by Marshall)?</t>
+        </is>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>Flast and Frothingham throw "very little light": Richardson didn't seek to invalidate a statute but claimed the Clause gives him a right to receive, and imposes an affirmative duty to supply, the report. The Flast nexus criteria were not "a litmus test" for all standing questions.</t>
+        </is>
+      </c>
+      <c r="F81" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>Professor's comment after Richardson: what did Halperin v. CIA hold?</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>A FOIA plaintiff who sought and was denied the CIA budget also lacked standing under the Statement and Account Clause; Richardson's holding covers all such challenges "whether by a mere taxpayer or by a FOIA plaintiff." 629 F.2d 144 (D.C. Cir. 1980). Prof asks: a fair interpretation?</t>
+        </is>
+      </c>
+      <c r="F82" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>United States v. Richardson (1974)</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>Did Richardson make a FOIA request for the CIA budget?</t>
+        </is>
+      </c>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>No (per the professor's comment).</t>
+        </is>
+      </c>
+      <c r="F83" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons: citation, author and lineup?</t>
+        </is>
+      </c>
+      <c r="E84" s="14" t="inlineStr">
+        <is>
+          <t>461 U.S. 95 (1983). Justice White for the Court, joined by Burger, Powell, Rehnquist and O'Connor. Marshall dissented, joined by Brennan, Blackmun and Stevens.</t>
+        </is>
+      </c>
+      <c r="F84" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>In what court did Lyons begin, and when?</t>
+        </is>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>U.S. District Court for the Central District of California; complaint filed February 7, 1977.</t>
+        </is>
+      </c>
+      <c r="F85" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>Lyons: who were the defendants, and what happened?</t>
+        </is>
+      </c>
+      <c r="E86" s="14" t="inlineStr">
+        <is>
+          <t>The City of Los Angeles and four of its police officers. On October 6, 1976 at 2 a.m., officers stopped Lyons for a traffic/vehicle code violation and, without provocation, applied a chokehold, rendering him unconscious and damaging his larynx.</t>
+        </is>
+      </c>
+      <c r="F86" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>Lyons: the two chokeholds at issue?</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>The "bar arm control" hold and the "carotid-artery control" hold.</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>Lyons: what did Counts I-IV, V and VI seek?</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>I-IV: damages against the officers and City. V (the focus): a preliminary and permanent injunction barring the holds. VI: a declaration that chokeholds absent threat of deadly force are per se unconstitutional.</t>
+        </is>
+      </c>
+      <c r="F88" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
+        <is>
+          <t>Lyons holding?</t>
+        </is>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>Lyons lacked standing to seek the injunction: past illegal choking may give standing for damages but does not establish "a real and immediate threat" he would again be stopped and illegally choked.</t>
+        </is>
+      </c>
+      <c r="F89" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>Lyons: the "incredible assertion" Lyons would have had to make?</t>
+        </is>
+      </c>
+      <c r="E90" s="14" t="inlineStr">
+        <is>
+          <t>That he would have another police encounter AND either (1) all LA police always choke any citizen they encounter, or (2) the City ordered or authorized officers to act in that manner.</t>
+        </is>
+      </c>
+      <c r="F90" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>Lyons: absent likelihood of future injury, Lyons is no more entitled to an injunction than whom?</t>
+        </is>
+      </c>
+      <c r="E91" s="14" t="inlineStr">
+        <is>
+          <t>"any other citizen of Los Angeles"; courts may not entertain claims by citizens who merely assert police practices are unconstitutional.</t>
+        </is>
+      </c>
+      <c r="F91" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>Marshall's dissent in Lyons: facts he emphasized?</t>
+        </is>
+      </c>
+      <c r="E92" s="14" t="inlineStr">
+        <is>
+          <t>Lyons, a 24-year-old Negro male, was stopped for a burned-out taillight, met with drawn revolvers, complained of pain from his keys, and within 5-10 seconds was choked until he blacked out; he urinated and defecated, then got a traffic citation and was released.</t>
+        </is>
+      </c>
+      <c r="F92" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>City of Los Angeles v. Lyons (1983)</t>
+        </is>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>Marshall's main doctrinal objection in Lyons?</t>
+        </is>
+      </c>
+      <c r="E93" s="14" t="inlineStr">
+        <is>
+          <t>The majority fragments standing by imposing a separate hurdle for each form of relief. Standing turns on the plaintiff's personal stake in the dispute, not in particular remedies; damages redress past injury and an injunction reduces future risk.</t>
+        </is>
+      </c>
+      <c r="F93" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>Davis, Administrative Law Treatise (2d ed. 1983)</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>Kenneth Culp Davis: how many standing cases, opinions and significant cases since 1978?</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>240 Supreme Court standing cases; more than 500 opinions including concurrences and dissents; 48 significant cases since 1978.</t>
+        </is>
+      </c>
+      <c r="F94" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>Davis, Administrative Law Treatise (2d ed. 1983)</t>
+        </is>
+      </c>
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>Argument</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>Davis: the "main failure" of standing law?</t>
+        </is>
+      </c>
+      <c r="E95" s="14" t="inlineStr">
+        <is>
+          <t>Not that the doors are opened too much or too little, but "the inconsistency, unreliability, and inordinate complexity."</t>
+        </is>
+      </c>
+      <c r="F95" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>Davis, Administrative Law Treatise (2d ed. 1983)</t>
+        </is>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>Professor's comment after Davis: what did Thole v. U.S. Bank say, and what does the professor ask?</t>
+        </is>
+      </c>
+      <c r="E96" s="14" t="inlineStr">
+        <is>
+          <t>"Courts sometimes make standing law more complicated than it needs to be." 140 S.Ct. 1615, 1622 (2020). Professor asks: "Any court in particular?"</t>
+        </is>
+      </c>
+      <c r="F96" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright: citation, author and lineup?</t>
+        </is>
+      </c>
+      <c r="E97" s="14" t="inlineStr">
+        <is>
+          <t>468 U.S. 737 (1984). Justice O'Connor for the Court, joined by Burger, White, Powell and Rehnquist. Dissents: Brennan; Stevens joined by Blackmun. Marshall took no part.</t>
+        </is>
+      </c>
+      <c r="F97" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Allen: what idea does the case-or-controversy requirement define for the Judicial Branch?</t>
+        </is>
+      </c>
+      <c r="E98" s="14" t="inlineStr">
+        <is>
+          <t>The idea of separation of powers (citing Valley Forge). "The law of Art. III standing is built on a single basic idea -- the idea of separation of powers."</t>
+        </is>
+      </c>
+      <c r="F98" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C99" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>Allen quotes Judge Bork's concurrence in which case, about doctrines clustering around Article III?</t>
+        </is>
+      </c>
+      <c r="E99" s="14" t="inlineStr">
+        <is>
+          <t>Vander Jagt v. O'Neill (D.C. Cir. 1983): standing, mootness, ripeness, political question relate to an idea "more than an intuition but less than a rigorous and explicit theory" about the limits on "an unelected, unrepresentative judiciary."</t>
+        </is>
+      </c>
+      <c r="F99" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C100" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D100" s="14" t="inlineStr">
+        <is>
+          <t>Allen: the three prudential ("judicially self-imposed") standing limits?</t>
+        </is>
+      </c>
+      <c r="E100" s="14" t="inlineStr">
+        <is>
+          <t>(1) General bar on raising another person's legal rights; (2) bar on adjudicating generalized grievances better addressed in the representative branches; (3) the complaint must fall within the zone of interests protected by the law invoked.</t>
+        </is>
+      </c>
+      <c r="F100" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>Allen: the constitutional core of standing?</t>
+        </is>
+      </c>
+      <c r="E101" s="14" t="inlineStr">
+        <is>
+          <t>"A plaintiff must allege personal injury fairly traceable to the defendant's allegedly unlawful conduct and likely to be redressed by the requested relief."</t>
+        </is>
+      </c>
+      <c r="F101" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>Allen: how must the injury be described (quoted terms)?</t>
+        </is>
+      </c>
+      <c r="E102" s="14" t="inlineStr">
+        <is>
+          <t>"Distinct and palpable" (Gladstone, quoting Warth), not "abstract," "conjectural" or "hypothetical" (Lyons); "fairly" traceable; relief "likely" (Simon).</t>
+        </is>
+      </c>
+      <c r="F102" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>Allen: the three questions the standing inquiry asks?</t>
+        </is>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
+        <is>
+          <t>Is the injury too abstract to be judicially cognizable? Is the line of causation too attenuated? Is the prospect of relief from a favorable ruling too speculative?</t>
+        </is>
+      </c>
+      <c r="F103" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>Allen: federal courts may exercise power only how (Chicago &amp; Grand Trunk R. Co. v. Wellman)?</t>
+        </is>
+      </c>
+      <c r="E104" s="14" t="inlineStr">
+        <is>
+          <t>"in the last resort, and as a necessity."</t>
+        </is>
+      </c>
+      <c r="F104" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="14" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>Allen: how can many standing questions be answered?</t>
+        </is>
+      </c>
+      <c r="E105" s="14" t="inlineStr">
+        <is>
+          <t>Chiefly by comparing the complaint's allegations with those in prior standing cases (citing Lyons).</t>
+        </is>
+      </c>
+      <c r="F105" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="14" t="inlineStr">
+        <is>
+          <t>Allen v. Wright (1984)</t>
+        </is>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>Warth v. Seldin, as quoted in Allen: "In essence the question of standing is..."?</t>
+        </is>
+      </c>
+      <c r="E106" s="14" t="inlineStr">
+        <is>
+          <t>"whether the litigant is entitled to have the court decide the merits of the dispute or of particular issues."</t>
+        </is>
+      </c>
+      <c r="F106" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C107" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife: citation and author?</t>
+        </is>
+      </c>
+      <c r="E107" s="14" t="inlineStr">
+        <is>
+          <t>504 U.S. 555 (1992). Justice Scalia for the Court (Parts I, II, III-A, IV), joined by Rehnquist, White, Kennedy, Souter, Thomas; Part III-B (redressability) was a plurality (Rehnquist, White, Thomas).</t>
+        </is>
+      </c>
+      <c r="F107" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C108" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: separate opinions?</t>
+        </is>
+      </c>
+      <c r="E108" s="14" t="inlineStr">
+        <is>
+          <t>Kennedy (joined by Souter) concurring in part and in the judgment; Stevens concurring in the judgment; Blackmun dissenting, with O'Connor.</t>
+        </is>
+      </c>
+      <c r="F108" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: what rule was challenged?</t>
+        </is>
+      </c>
+      <c r="E109" s="14" t="inlineStr">
+        <is>
+          <t>A rule by the Secretary of the Interior interpreting ESA § 7(a)(2) (16 U.S.C. § 1536(a)(2)) to require consultation only for actions in the United States or on the high seas.</t>
+        </is>
+      </c>
+      <c r="F109" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>ESA § 7(a)(2) requires what?</t>
+        </is>
+      </c>
+      <c r="E110" s="14" t="inlineStr">
+        <is>
+          <t>Each federal agency, in consultation with the Secretary, must insure that any action it authorizes, funds or carries out is not likely to jeopardize endangered or threatened species or destroy critical habitat.</t>
+        </is>
+      </c>
+      <c r="F110" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C111" s="14" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: history of the regulation?</t>
+        </is>
+      </c>
+      <c r="E111" s="14" t="inlineStr">
+        <is>
+          <t>1978: FWS and NMFS joint regulation extended § 7(a)(2) to foreign nations. Interior began reexamining it the next year; a revised regulation limiting it to the U.S. and high seas was proposed in 1983 and promulgated in 1986.</t>
+        </is>
+      </c>
+      <c r="F111" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C112" s="14" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: procedural history?</t>
+        </is>
+      </c>
+      <c r="E112" s="14" t="inlineStr">
+        <is>
+          <t>District Court dismissed for lack of standing; Eighth Circuit reversed (divided). On remand the District Court denied the Secretary's SJ motion and granted respondents' merits motion; Eighth Circuit affirmed; cert granted. Supreme Court reversed and remanded.</t>
+        </is>
+      </c>
+      <c r="F112" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C113" s="14" t="inlineStr">
+        <is>
+          <t>Separation</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: what examples show "case" and "controversy" can name non-judicial matters?</t>
+        </is>
+      </c>
+      <c r="E113" s="14" t="inlineStr">
+        <is>
+          <t>An executive inquiry ("the Hoffa case") and a legislative dispute ("the Smoot-Hawley controversy"). Scalia also quotes Madison's Federalist No. 48 that the judiciary is described by "landmarks still less uncertain."</t>
+        </is>
+      </c>
+      <c r="F113" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C114" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: the "irreducible constitutional minimum" of standing?</t>
+        </is>
+      </c>
+      <c r="E114" s="14" t="inlineStr">
+        <is>
+          <t>(1) Injury in fact: invasion of a legally protected interest that is (a) concrete and particularized and (b) actual or imminent, not conjectural or hypothetical; (2) causation: fairly traceable to the defendant, not an independent third party; (3) redressability: "likely," not "speculative."</t>
+        </is>
+      </c>
+      <c r="F114" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C115" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>Lujan footnote 1: what does "particularized" mean?</t>
+        </is>
+      </c>
+      <c r="E115" s="14" t="inlineStr">
+        <is>
+          <t>"the injury must affect the plaintiff in a personal and individual way."</t>
+        </is>
+      </c>
+      <c r="F115" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: who bears the burden of standing, and how?</t>
+        </is>
+      </c>
+      <c r="E116" s="14" t="inlineStr">
+        <is>
+          <t>The party invoking jurisdiction; the elements are not mere pleading requirements, so each must be supported with the manner and degree of evidence required at the successive stages of litigation.</t>
+        </is>
+      </c>
+      <c r="F116" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="14" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D117" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: object of government action vs. regulation of someone else?</t>
+        </is>
+      </c>
+      <c r="E117" s="14" t="inlineStr">
+        <is>
+          <t>If the plaintiff is the object, there is ordinarily little question of injury and redress. If the injury arises from regulation (or non-regulation) of a third party, standing is "not precluded" but "substantially more difficult" to establish.</t>
+        </is>
+      </c>
+      <c r="F117" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C118" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: Joyce Kelly's affidavit?</t>
+        </is>
+      </c>
+      <c r="E118" s="14" t="inlineStr">
+        <is>
+          <t>She traveled to Egypt in 1986, observed the traditional habitat of the endangered Nile crocodile, and intends to return; harmed by the American role in rehabilitating the Aswan High Dam and developing Egypt's Master Water Plan.</t>
+        </is>
+      </c>
+      <c r="F118" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="14" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: Amy Skilbred's affidavit and deposition?</t>
+        </is>
+      </c>
+      <c r="E119" s="14" t="inlineStr">
+        <is>
+          <t>She visited Sri Lanka in 1981 and observed habitat of the Asian elephant and leopard at the AID-funded Mahaweli project site (but saw none). Asked when she would return: "There is a civil war going on right now. I don't know. Not next year, I will say. In the future."</t>
+        </is>
+      </c>
+      <c r="F119" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C120" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D120" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: why were Kelly and Skilbred's intentions to return insufficient?</t>
+        </is>
+      </c>
+      <c r="E120" s="14" t="inlineStr">
+        <is>
+          <t>"Some day" intentions, without concrete plans or any specification of when, do not show "actual or imminent" injury. Past visits prove nothing (citing Lyons on past exposure).</t>
+        </is>
+      </c>
+      <c r="F120" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C121" s="14" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>Lujan footnote 2: why reject the dissent's "soon"?</t>
+        </is>
+      </c>
+      <c r="E121" s="14" t="inlineStr">
+        <is>
+          <t>If "soon" means imminent, a mere intent to return some day fails factually; if it means "in this lifetime," it departs from precedent. Imminence ensures injury is "certainly impending," especially where the acts making the injury happen are partly within the plaintiff's own control.</t>
+        </is>
+      </c>
+      <c r="F121" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C122" s="14" t="inlineStr">
+        <is>
+          <t>Nexus theories</t>
+        </is>
+      </c>
+      <c r="D122" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: the "ecosystem nexus" theory and why rejected?</t>
+        </is>
+      </c>
+      <c r="E122" s="14" t="inlineStr">
+        <is>
+          <t>Anyone using any part of a "contiguous ecosystem" affected by a funded activity has standing. Rejected under National Wildlife Federation: the plaintiff must use the area affected, not an area roughly "in the vicinity."</t>
+        </is>
+      </c>
+      <c r="F122" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="14" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C123" s="14" t="inlineStr">
+        <is>
+          <t>Nexus theories</t>
+        </is>
+      </c>
+      <c r="D123" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: the "animal nexus" and "vocational nexus" theories?</t>
+        </is>
+      </c>
+      <c r="E123" s="14" t="inlineStr">
+        <is>
+          <t>Anyone interested in seeing the endangered animals anywhere, or anyone with a professional interest in them, could sue. Scalia: then anyone who sees, or keeps, Asian elephants in the Bronx Zoo could sue over Sri Lanka. "This is beyond all reason."</t>
+        </is>
+      </c>
+      <c r="F123" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C124" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: standing is not what (quoting SCRAP)?</t>
+        </is>
+      </c>
+      <c r="E124" s="14" t="inlineStr">
+        <is>
+          <t>"an ingenious academic exercise in the conceivable."</t>
+        </is>
+      </c>
+      <c r="F124" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="14" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C125" s="14" t="inlineStr">
+        <is>
+          <t>Redressability</t>
+        </is>
+      </c>
+      <c r="D125" s="14" t="inlineStr">
+        <is>
+          <t>Lujan Part III-B (plurality): why was redressability lacking?</t>
+        </is>
+      </c>
+      <c r="E125" s="14" t="inlineStr">
+        <is>
+          <t>The funding agencies were not parties and arguably not bound by the Secretary's regulation (the Solicitor General repudiated that it binds them); and the agencies supply only a fraction of foreign project funding (AID gave less than 10% of Mahaweli's).</t>
+        </is>
+      </c>
+      <c r="F125" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C126" s="14" t="inlineStr">
+        <is>
+          <t>Redressability</t>
+        </is>
+      </c>
+      <c r="D126" s="14" t="inlineStr">
+        <is>
+          <t>Lujan footnote 5: response to Justice Stevens's point that agencies would follow a Supreme Court ruling?</t>
+        </is>
+      </c>
+      <c r="E126" s="14" t="inlineStr">
+        <is>
+          <t>Standing is determined as of the commencement of suit, when it could not be known the case would reach the Supreme Court.</t>
+        </is>
+      </c>
+      <c r="F126" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C127" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D127" s="14" t="inlineStr">
+        <is>
+          <t>Lujan Part IV: what did the Eighth Circuit hold about "procedural injury"?</t>
+        </is>
+      </c>
+      <c r="E127" s="14" t="inlineStr">
+        <is>
+          <t>That the ESA citizen-suit provision (16 U.S.C. § 1540(g), "any person may commence a civil suit") gave all persons a procedural right to consultation. The Court rejected this "abstract, self-contained, noninstrumental 'right'" to have the Executive observe procedures.</t>
+        </is>
+      </c>
+      <c r="F127" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C128" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D128" s="14" t="inlineStr">
+        <is>
+          <t>Lujan footnote 7: when may a procedural-rights plaintiff relax redressability and immediacy?</t>
+        </is>
+      </c>
+      <c r="E128" s="14" t="inlineStr">
+        <is>
+          <t>When the procedure protects his concrete interests: e.g., one living adjacent to a proposed federally licensed dam may challenge the failure to prepare an environmental impact statement, though he can't show the EIS would change the outcome and the dam is years away.</t>
+        </is>
+      </c>
+      <c r="F128" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="14" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C129" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D129" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: which earlier generalized-grievance cases did Scalia cite?</t>
+        </is>
+      </c>
+      <c r="E129" s="14" t="inlineStr">
+        <is>
+          <t>Fairchild v. Hughes (Brandeis; challenge to the Nineteenth Amendment's ratification process); Massachusetts v. Mellon; Richardson; Allen and Valley Forge; Whitmore (citizen suit to stop an execution).</t>
+        </is>
+      </c>
+      <c r="F129" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C130" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D130" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: which constitutional duty would Congress transfer to courts by converting the public interest into an individual right?</t>
+        </is>
+      </c>
+      <c r="E130" s="14" t="inlineStr">
+        <is>
+          <t>The President's duty to "take Care that the Laws be faithfully executed" (Art. II, § 3); courts would become "virtually continuing monitors of the wisdom and soundness of Executive action" (Allen, quoting Laird v. Tatum).</t>
+        </is>
+      </c>
+      <c r="F130" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="14" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C131" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D131" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: what line from Marbury did Scalia quote?</t>
+        </is>
+      </c>
+      <c r="E131" s="14" t="inlineStr">
+        <is>
+          <t>"The province of the court... is, solely, to decide on the rights of individuals." Vindicating the public interest is the function of Congress and the Chief Executive.</t>
+        </is>
+      </c>
+      <c r="F131" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C132" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D132" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: does the source of the right (Constitution vs. statute) matter?</t>
+        </is>
+      </c>
+      <c r="E132" s="14" t="inlineStr">
+        <is>
+          <t>"There is absolutely no basis for making the Article III inquiry turn on the source of the asserted right." In suits against the Government, at least, the concrete injury requirement must remain.</t>
+        </is>
+      </c>
+      <c r="F132" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C133" s="14" t="inlineStr">
+        <is>
+          <t>Procedural injury</t>
+        </is>
+      </c>
+      <c r="D133" s="14" t="inlineStr">
+        <is>
+          <t>Lujan: how did Scalia reconcile Warth/Linda R.S. ("statutes creating legal rights, the invasion of which creates standing")?</t>
+        </is>
+      </c>
+      <c r="E133" s="14" t="inlineStr">
+        <is>
+          <t>Those examples elevated concrete, de facto injuries previously inadequate in law (living in an integrated community; marketing free of competition). Broadening categories of injury differs from abandoning the requirement that the plaintiff himself be injured (Sierra Club).</t>
+        </is>
+      </c>
+      <c r="F133" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C134" s="14" t="inlineStr">
+        <is>
+          <t>Concurrence</t>
+        </is>
+      </c>
+      <c r="D134" s="14" t="inlineStr">
+        <is>
+          <t>Kennedy's concurrence in Lujan (with Souter)?</t>
+        </is>
+      </c>
+      <c r="E134" s="14" t="inlineStr">
+        <is>
+          <t>Agreed the affiants weren't "among the injured"; noted it "may seem trivial" to require airline tickets or a date certain but they didn't use the sites regularly; would not foreclose nexus theories in other circumstances (Japan Whaling); would not reach redressability (Part III-B).</t>
+        </is>
+      </c>
+      <c r="F134" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C135" s="14" t="inlineStr">
+        <is>
+          <t>Concurrence</t>
+        </is>
+      </c>
+      <c r="D135" s="14" t="inlineStr">
+        <is>
+          <t>Stevens's concurrence in the judgment in Lujan?</t>
+        </is>
+      </c>
+      <c r="E135" s="14" t="inlineStr">
+        <is>
+          <t>He concurred because Congress did not intend § 7(a)(2) consultation to apply abroad (the merits), but disagreed that the injury was not "imminent" or not "redressable."</t>
+        </is>
+      </c>
+      <c r="F135" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C136" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D136" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun's dissent in Lujan: summary-judgment argument?</t>
+        </is>
+      </c>
+      <c r="E136" s="14" t="inlineStr">
+        <is>
+          <t>Respondents needed only a "genuine issue" of material fact (Rule 56(c)), which the Court never mentions; it confused the evidentiary burden (Rule 56(e)) with the standard of proof.</t>
+        </is>
+      </c>
+      <c r="F136" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C137" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D137" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun in Lujan: on concrete plans and plane tickets?</t>
+        </is>
+      </c>
+      <c r="E137" s="14" t="inlineStr">
+        <is>
+          <t>Requiring concrete plans demands "an empty formality"; nothing prevents Kelly or Skilbred from buying plane tickets. Unlike Lyons, harm here did not depend on third parties' actions.</t>
+        </is>
+      </c>
+      <c r="F137" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C138" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun in Lujan: "Three-Card Monte" and the $170 million point?</t>
+        </is>
+      </c>
+      <c r="E138" s="14" t="inlineStr">
+        <is>
+          <t>The Government cannot play "Three-Card Monte" with agencies' authority after the Secretary had said his rules bind them. AID's "fraction" of Mahaweli funding was $170 million, large for a country of 16 million with GNP under $6 billion (1986).</t>
+        </is>
+      </c>
+      <c r="F138" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="14" t="inlineStr">
+        <is>
+          <t>Lujan v. Defenders of Wildlife (1992)</t>
+        </is>
+      </c>
+      <c r="C139" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>Blackmun's closing in Lujan?</t>
+        </is>
+      </c>
+      <c r="E139" s="14" t="inlineStr">
+        <is>
+          <t>He cannot join "a slash-and-burn expedition through the law of environmental standing," quoting Marbury: "the very essence of civil liberty certainly consists in the right of every individual to claim the protection of the laws, whenever he receives an injury."</t>
+        </is>
+      </c>
+      <c r="F139" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C140" s="14" t="inlineStr">
+        <is>
+          <t>Basics</t>
+        </is>
+      </c>
+      <c r="D140" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins: citation, author and lineup?</t>
+        </is>
+      </c>
+      <c r="E140" s="14" t="inlineStr">
+        <is>
+          <t>524 U.S. 11 (1998). Justice Breyer for the Court, joined by Rehnquist, Stevens, Kennedy, Souter and Ginsburg. Scalia dissented, joined by O'Connor and Thomas.</t>
+        </is>
+      </c>
+      <c r="F140" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="14" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C141" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D141" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins: what did the FEC decide?</t>
+        </is>
+      </c>
+      <c r="E141" s="14" t="inlineStr">
+        <is>
+          <t>That the American Israel Public Affairs Committee (AIPAC) was not a "political committee" under the Federal Election Campaign Act of 1971, so it need not disclose its membership, contributions and expenditures.</t>
+        </is>
+      </c>
+      <c r="F141" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="14" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C142" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D142" s="14" t="inlineStr">
+        <is>
+          <t>Who were the respondents in Akins, and what did the Court hold?</t>
+        </is>
+      </c>
+      <c r="E142" s="14" t="inlineStr">
+        <is>
+          <t>A group of voters; they had standing to challenge the FEC's determination. Remanded.</t>
+        </is>
+      </c>
+      <c r="F142" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="14" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C143" s="14" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="D143" s="14" t="inlineStr">
+        <is>
+          <t>Akins: which of the two certiorari questions did the Court answer?</t>
+        </is>
+      </c>
+      <c r="E143" s="14" t="inlineStr">
+        <is>
+          <t>Only the first (standing). It did not decide whether a group spending over $1,000 that is not candidate-controlled and lacks the major purpose of electing candidates is a "political committee."</t>
+        </is>
+      </c>
+      <c r="F143" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="14" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C144" s="14" t="inlineStr">
+        <is>
+          <t>Prudential</t>
+        </is>
+      </c>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>Akins: why were prudential standing requirements satisfied?</t>
+        </is>
+      </c>
+      <c r="E144" s="14" t="inlineStr">
+        <is>
+          <t>FECA lets "any person who believes a violation... has occurred" file a complaint (§ 437g(a)(1)) and "any party aggrieved" by dismissal petition a district court (§ 437g(a)(8)(A)); Congress meant to protect voters like respondents.</t>
+        </is>
+      </c>
+      <c r="F144" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="14" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C145" s="14" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="D145" s="14" t="inlineStr">
+        <is>
+          <t>Akins: what was the injury in fact?</t>
+        </is>
+      </c>
+      <c r="E145" s="14" t="inlineStr">
+        <is>
+          <t>Inability to obtain information (AIPAC donor/member lists, campaign contributions and expenditures) that the statute arguably requires be made public, which would help them evaluate candidates.</t>
+        </is>
+      </c>
+      <c r="F145" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="14" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C146" s="14" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="D146" s="14" t="inlineStr">
+        <is>
+          <t>Akins: precedents for informational injury?</t>
+        </is>
+      </c>
+      <c r="E146" s="14" t="inlineStr">
+        <is>
+          <t>Public Citizen v. Department of Justice (Federal Advisory Committee Act) and Havens Realty Corp. v. Coleman (information about housing availability).</t>
+        </is>
+      </c>
+      <c r="F146" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="14" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C147" s="14" t="inlineStr">
+        <is>
+          <t>Richardson</t>
+        </is>
+      </c>
+      <c r="D147" s="14" t="inlineStr">
+        <is>
+          <t>How did Akins distinguish Richardson?</t>
+        </is>
+      </c>
+      <c r="E147" s="14" t="inlineStr">
+        <is>
+          <t>No constitutional "logical nexus" requirement applies here; instead a statute seeks to protect individuals like respondents. And Richardson focused on taxpayer standing, not voter standing.</t>
+        </is>
+      </c>
+      <c r="F147" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="14" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C148" s="14" t="inlineStr">
+        <is>
+          <t>Generalized grievance</t>
+        </is>
+      </c>
+      <c r="D148" s="14" t="inlineStr">
+        <is>
+          <t>Akins: when does a widely shared injury still count?</t>
+        </is>
+      </c>
+      <c r="E148" s="14" t="inlineStr">
+        <is>
+          <t>Generalized-grievance language appears where harm is both widely shared and "abstract and indefinite" (e.g., "common concern for obedience to law"). Where harm is concrete, though widely shared (mass tort, voting-rights interference), it is injury in fact.</t>
+        </is>
+      </c>
+      <c r="F148" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="14" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C149" s="14" t="inlineStr">
+        <is>
+          <t>Key phrases</t>
+        </is>
+      </c>
+      <c r="D149" s="14" t="inlineStr">
+        <is>
+          <t>Akins: how did the Court describe the informational injury here?</t>
+        </is>
+      </c>
+      <c r="E149" s="14" t="inlineStr">
+        <is>
+          <t>"directly related to voting, the most basic of political rights," and sufficiently concrete and specific that its being widely shared does not deprive Congress of power to authorize suit.</t>
+        </is>
+      </c>
+      <c r="F149" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C150" s="14" t="inlineStr">
+        <is>
+          <t>Causation</t>
+        </is>
+      </c>
+      <c r="D150" s="14" t="inlineStr">
+        <is>
+          <t>Akins: does the FEC's discretion defeat traceability/redressability?</t>
+        </is>
+      </c>
+      <c r="E150" s="14" t="inlineStr">
+        <is>
+          <t>No. Even if the FEC might reach the same result lawfully, a court that finds the agency misinterpreted the law sets aside and remands, "like a new jury after a mistrial."</t>
+        </is>
+      </c>
+      <c r="F150" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C151" s="14" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D151" s="14" t="inlineStr">
+        <is>
+          <t>Akins: why didn't Heckler v. Chaney bar review of the FEC's non-enforcement?</t>
+        </is>
+      </c>
+      <c r="E151" s="14" t="inlineStr">
+        <is>
+          <t>Heckler held enforcement decisions traditionally "committed to agency discretion" under the APA, but FECA "explicitly indicates the contrary."</t>
+        </is>
+      </c>
+      <c r="F151" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="14" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C152" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D152" s="14" t="inlineStr">
+        <is>
+          <t>Scalia's dissent in Akins: statutory argument?</t>
+        </is>
+      </c>
+      <c r="E152" s="14" t="inlineStr">
+        <is>
+          <t>FECA distinguishes "any person" who may complain from a "party aggrieved" who may sue; respondents complain not of refusal to provide information but of refusal to enforce against a third party. Constitutional doubt also counsels a narrow reading.</t>
+        </is>
+      </c>
+      <c r="F152" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="14" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C153" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D153" s="14" t="inlineStr">
+        <is>
+          <t>Scalia in Akins: timing of the citizen-suit provision?</t>
+        </is>
+      </c>
+      <c r="E153" s="14" t="inlineStr">
+        <is>
+          <t>It was enacted two years after Richardson, which gave Congress every reason to think a voter's informational interest was constitutionally inadequate.</t>
+        </is>
+      </c>
+      <c r="F153" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="14" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C154" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D154" s="14" t="inlineStr">
+        <is>
+          <t>Scalia in Akins: what did the majority reduce Richardson to, and what did he call the distinction?</t>
+        </is>
+      </c>
+      <c r="E154" s="14" t="inlineStr">
+        <is>
+          <t>"from a landmark constitutional holding to a curio"; the taxpayer/voter distinction is "silly." He mocks the "unaccustomed ineptitude" of the ACLU Foundation (which litigated Richardson) for not refiling as voters.</t>
+        </is>
+      </c>
+      <c r="F154" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="14" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C155" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D155" s="14" t="inlineStr">
+        <is>
+          <t>Scalia in Akins: the tort-victim illustration?</t>
+        </is>
+      </c>
+      <c r="E155" s="14" t="inlineStr">
+        <is>
+          <t>Mass-tort and voting injuries are widely shared but particularized: "One tort victim suffers a burnt leg, another a burnt arm." A generalized grievance is undifferentiated, like Richardson's and Akins's identical lack of information.</t>
+        </is>
+      </c>
+      <c r="F155" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="14" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C156" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D156" s="14" t="inlineStr">
+        <is>
+          <t>Scalia in Akins: the separation-of-powers conclusion?</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
+        <is>
+          <t>Letting any voter compel Executive enforcement transfers the "take Care" duty (Art. II, § 3) to the courts; Congress could authorize anyone to manage enforcement of any law requiring "the filing and public availability of a piece of paper."</t>
+        </is>
+      </c>
+      <c r="F156" s="97" t="inlineStr">
+        <is>
+          <t>Must-know</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="14" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="14" t="inlineStr">
+        <is>
+          <t>FEC v. Akins (1998)</t>
+        </is>
+      </c>
+      <c r="C157" s="14" t="inlineStr">
+        <is>
+          <t>Dissent</t>
+        </is>
+      </c>
+      <c r="D157" s="14" t="inlineStr">
+        <is>
+          <t>Scalia in Akins footnote 1: Schlesinger v. Reservists?</t>
+        </is>
+      </c>
+      <c r="E157" s="14" t="inlineStr">
+        <is>
+          <t>Decided the same day as Richardson: "the Flast nexus test is not applicable where the taxing and spending power is not challenged."</t>
+        </is>
+      </c>
+      <c r="F157" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F157"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>